<commit_message>
feat(scans): roll validated v4 rules out to all 10 demo servers
All 10 scans now scan-rules-v4 (ONE-CALL rule, breadth limits, sensitivity
anchors). Consistency findings 151->80 (I1/I3/I4 zero everywhere; residual is
the documented metadata-op limitation). ranked_calls regenerated; bundle
reports/all_scans_v4.zip.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/scan/calendar_cbg.xlsx
+++ b/reports/scan/calendar_cbg.xlsx
@@ -41,12 +41,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFCC99"/>
+        <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
+        <fgColor rgb="00FFCC99"/>
       </patternFill>
     </fill>
     <fill>
@@ -517,50 +517,50 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
           <t>16</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>24</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="K2" s="3" t="inlineStr">
         <is>
           <t>24</t>
         </is>
@@ -579,57 +579,57 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>12</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>12</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>4</t>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="L3" s="4" t="inlineStr">
-        <is>
-          <t>60</t>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>36</t>
         </is>
       </c>
     </row>
@@ -639,52 +639,52 @@
           <t>executive</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
           <t>16</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>24</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>24</t>
         </is>
@@ -701,59 +701,59 @@
           <t>recruiting</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t>24</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="K5" s="3" t="inlineStr">
         <is>
           <t>24</t>
         </is>
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>48</t>
         </is>
       </c>
     </row>
@@ -763,59 +763,59 @@
           <t>contacts</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>16</t>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>20</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>20</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="J6" s="4" t="inlineStr">
-        <is>
-          <t>48</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>24</t>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>30</t>
         </is>
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>60</t>
         </is>
       </c>
     </row>
@@ -825,59 +825,59 @@
           <t>holidays</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>8</t>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>4</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="I7" s="3" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="J7" s="3" t="inlineStr">
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>12</t>
-        </is>
-      </c>
-      <c r="K7" s="3" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="L7" s="2" t="inlineStr">
-        <is>
-          <t>24</t>
         </is>
       </c>
     </row>
@@ -1046,7 +1046,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17">
@@ -1076,7 +1076,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="20">
@@ -1086,7 +1086,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(scans): roll v6 rules (reach-is-a-count) out to all 10 servers
All 10 now scan-rules-v6. ranked_calls + xlsx/matrix regenerated. 317 tests pass.
Judge-driven improvement converged: per-primitive impact 92% / sensitivity 90% /
blast 76%, heatmap coherence github 85% / corp 87%, blast drift 1/1.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/scan/calendar_cbg.xlsx
+++ b/reports/scan/calendar_cbg.xlsx
@@ -41,12 +41,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
+        <fgColor rgb="00FFCC99"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFCC99"/>
+        <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
     <fill>
@@ -517,50 +517,50 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
+          <t>16</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>24</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>24</t>
         </is>
@@ -577,17 +577,17 @@
           <t>team</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>12</t>
         </is>
@@ -597,37 +597,37 @@
           <t>3</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>18</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>18</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>36</t>
         </is>
@@ -639,59 +639,59 @@
           <t>executive</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>24</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>24</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>48</t>
         </is>
       </c>
     </row>
@@ -701,52 +701,52 @@
           <t>recruiting</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="J5" s="3" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>24</t>
         </is>
       </c>
-      <c r="K5" s="3" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>24</t>
         </is>
@@ -763,52 +763,52 @@
           <t>contacts</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="J6" s="3" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="K6" s="3" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>30</t>
         </is>
@@ -865,17 +865,17 @@
           <t>4</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="J7" s="3" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="K7" s="3" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="L7" s="3" t="inlineStr">
         <is>
           <t>12</t>
         </is>

</xml_diff>